<commit_message>
rework and split the reversal figures into landscape, trajectory, and fry
</commit_message>
<xml_diff>
--- a/04_Figures/F04_Reversal/c_data/F04_supplementary.xlsx
+++ b/04_Figures/F04_Reversal/c_data/F04_supplementary.xlsx
@@ -320,7 +320,7 @@
     <t xml:space="preserve">REACTOME_MHC_CLASS_II_ANTIGEN_PRESENTATION</t>
   </si>
   <si>
-    <t xml:space="preserve">Mhc Class Ii Antigen Presentation</t>
+    <t xml:space="preserve">MHC Class II Antigen Presentation</t>
   </si>
   <si>
     <t xml:space="preserve">REACTOME_BRANCHED_CHAIN_AMINO_ACID_CATABOLISM</t>
@@ -2543,7 +2543,7 @@
     <t xml:space="preserve">GOSLIM_TRNA_METABOLIC_PROCESS</t>
   </si>
   <si>
-    <t xml:space="preserve">Trna Metabolic Process</t>
+    <t xml:space="preserve">tRNA Metabolic Process</t>
   </si>
   <si>
     <t xml:space="preserve">HALLMARK_EPITHELIAL_MESENCHYMAL_TRANSITION</t>
@@ -5417,13 +5417,13 @@
     <t xml:space="preserve">KEGG</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference Mitochondrial Complex Ucp1 In Thermogenesis</t>
+    <t xml:space="preserve">Mitochondrial Complex Ucp1 In Thermogenesis</t>
   </si>
   <si>
     <t xml:space="preserve">KEGG_MEDICUS_REFERENCE_ELECTRON_TRANSFER_IN_COMPLEX_I</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference Electron Transfer In Complex I</t>
+    <t xml:space="preserve">Electron Transfer In Complex I</t>
   </si>
   <si>
     <t xml:space="preserve">REACTOME_COMPLEX_I_BIOGENESIS</t>
@@ -5507,13 +5507,13 @@
     <t xml:space="preserve">REACTOME_CYTOSOLIC_TRNA_AMINOACYLATION</t>
   </si>
   <si>
-    <t xml:space="preserve">Cytosolic Trna Aminoacylation</t>
+    <t xml:space="preserve">Cytosolic tRNA Aminoacylation</t>
   </si>
   <si>
     <t xml:space="preserve">REACTOME_COMPLEX_IV_ASSEMBLY</t>
   </si>
   <si>
-    <t xml:space="preserve">Complex Iv Assembly</t>
+    <t xml:space="preserve">Complex IV Assembly</t>
   </si>
   <si>
     <t xml:space="preserve">REACTOME_GLYCOGEN_METABOLISM</t>

</xml_diff>